<commit_message>
Estimativas de custos: inclusão de apis azure e totais de tokens p/ segundo consumidos
</commit_message>
<xml_diff>
--- a/artefatos/dados_coletados/cenarios.xlsx
+++ b/artefatos/dados_coletados/cenarios.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="agencias" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t xml:space="preserve">Território</t>
   </si>
@@ -84,6 +84,120 @@
   </si>
   <si>
     <t xml:space="preserve">SerproLLM: Speech Service e gemma-4-31b</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APIS MS Azure: Fast-Transcribe e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">GPT-5.6-luna</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">APIS MS Azure: Fast-Transcribe e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GPT-5-mini</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">APIS MS Azure: Fast-Transcribe e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GPT-5-chat</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">APIS MS Azure: Fast-Transcribe e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GPT-5.2-chat</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">APIS MS Azure: Fast-Transcribe e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GPT-5.6-terra</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">APIS MS Azure: Fast-Transcribe e </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GPT-5.6-sol</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -93,11 +207,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -118,6 +233,12 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -162,21 +283,29 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -305,67 +434,67 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="55.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="30.66"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="58" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="46.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>3562</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="4" t="n">
         <v>4553167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2649</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>8175000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>1385.685</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>2982818</v>
       </c>
     </row>
@@ -385,140 +514,230 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="37.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>0.24</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>0.24</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>0.24</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>1.5</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>7.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>0.11</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>0.23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>0.21</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>0.62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>0.2996</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>1.19845</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>0.494</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>2.9411</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <v>0.1597</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>0.67911</v>
       </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0"/>
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+      <c r="D16" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>